<commit_message>
major humongous update -- new search data from MQ v2.8.0.0
</commit_message>
<xml_diff>
--- a/Dependencies/Analysis_Outputs/Ping_2018/N_samples_in_datasets.xlsx
+++ b/Dependencies/Analysis_Outputs/Ping_2018/N_samples_in_datasets.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,7 +511,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>fcb2</t>
+          <t>fcb1</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -524,7 +524,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>fcb3</t>
+          <t>fcb2</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -537,7 +537,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>fcb4</t>
+          <t>fcb3</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -550,10 +550,23 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>fcb4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>fcb5</t>
         </is>
       </c>
-      <c r="C10" t="n">
+      <c r="C11" t="n">
         <v>10</v>
       </c>
     </row>

</xml_diff>